<commit_message>
Fill Rally x Antseed KOL list with real roster (14 KOLs, $5,400)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P3jSSdGqNpHohJRWxCoL15
</commit_message>
<xml_diff>
--- a/kol-tracker/partners/Rally_x_Antseed_KOL_List.xlsx
+++ b/kol-tracker/partners/Rally_x_Antseed_KOL_List.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
   <si>
     <t xml:space="preserve">Rally x Antseed — KOL Campaign</t>
   </si>
@@ -71,7 +71,7 @@
     <t xml:space="preserve">Confirmed budget ($)</t>
   </si>
   <si>
-    <t xml:space="preserve">Yellow cells are editable. Rows marked '(example)' in the KOL List are placeholders — replace with real KOLs.</t>
+    <t xml:space="preserve">Yellow cells are editable. Followers, region, deliverables and status are pending — fill them in as they get confirmed.</t>
   </si>
   <si>
     <t xml:space="preserve">Rally x Antseed — KOL List</t>
@@ -113,67 +113,130 @@
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
-    <t xml:space="preserve">Ana Example</t>
-  </si>
-  <si>
-    <t xml:space="preserve">@ana_web3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://x.com/ana_web3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LATAM / ES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DeFi threads</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 posts + 1 thread</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proposed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(example) replace</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bruno Example</t>
-  </si>
-  <si>
-    <t xml:space="preserve">@brunocripto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://x.com/brunocripto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Global / EN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trading content</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 posts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carla Example</t>
-  </si>
-  <si>
-    <t xml:space="preserve">@carla_defi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://x.com/carla_defi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEA / EN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ecosystem reviews</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 thread + 1 space</t>
+    <t xml:space="preserve">Gujjuiixi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Gujjuiixi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/Gujjuiixi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rakib_web3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Rakib_web3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/Rakib_web3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notjazii</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Notjazii</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/Notjazii</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hasantoxr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Hasantoxr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/Hasantoxr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tuge8888</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Tuge8888</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/Tuge8888</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alphabatcher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Alphabatcher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/Alphabatcher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zijing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Zijing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/Zijing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zaimiri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Zaimiri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/Zaimiri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Afrochicksnft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Afrochicksnft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/Afrochicksnft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MrTimister</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@MrTimister</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/MrTimister</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MedusaOnChain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@MedusaOnChain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/MedusaOnChain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CrypSaf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@CrypSaf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/CrypSaf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horkays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Horkays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/Horkays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jgonzalezferrer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@jgonzalezferrer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://x.com/jgonzalezferrer</t>
   </si>
 </sst>
 </file>
@@ -709,7 +772,7 @@
       </c>
       <c r="C11" s="6" t="n">
         <f aca="false">COUNTA('KOL List'!$B$4:$B$200)</f>
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -718,7 +781,7 @@
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">COUNTIF('KOL List'!$K$4:$K$200,"Confirmed")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -727,7 +790,7 @@
       </c>
       <c r="C13" s="6" t="n">
         <f aca="false">SUM('KOL List'!$E$4:$E$200)</f>
-        <v>181500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -736,7 +799,7 @@
       </c>
       <c r="C14" s="7" t="n">
         <f aca="false">SUM('KOL List'!$J$4:$J$200)</f>
-        <v>1600</v>
+        <v>5400</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -745,7 +808,7 @@
       </c>
       <c r="C15" s="7" t="n">
         <f aca="false">SUMIF('KOL List'!$K$4:$K$200,"Confirmed",'KOL List'!$J$4:$J$200)</f>
-        <v>450</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -843,31 +906,19 @@
       <c r="D4" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="11" t="n">
-        <v>125000</v>
-      </c>
+      <c r="E4" s="11"/>
       <c r="F4" s="12" t="str">
         <f aca="false">IF(E4="","",IF(E4&lt;10000,"Micro",IF(E4&lt;100000,"Mid","Macro")))</f>
-        <v>Macro</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>35</v>
-      </c>
+        <v/>
+      </c>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
       <c r="J4" s="13" t="n">
-        <v>900</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>37</v>
-      </c>
+        <v>300</v>
+      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="n">
@@ -875,39 +926,27 @@
         <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>48000</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="E5" s="11"/>
       <c r="F5" s="12" t="str">
         <f aca="false">IF(E5="","",IF(E5&lt;10000,"Micro",IF(E5&lt;100000,"Mid","Macro")))</f>
-        <v>Mid</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>43</v>
-      </c>
+        <v/>
+      </c>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
       <c r="J5" s="13" t="n">
-        <v>450</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>37</v>
-      </c>
+        <v>300</v>
+      </c>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="n">
@@ -915,48 +954,42 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>8500</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="E6" s="11"/>
       <c r="F6" s="12" t="str">
         <f aca="false">IF(E6="","",IF(E6&lt;10000,"Micro",IF(E6&lt;100000,"Mid","Macro")))</f>
-        <v>Micro</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>50</v>
-      </c>
+        <v/>
+      </c>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
       <c r="J6" s="13" t="n">
-        <v>250</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>37</v>
-      </c>
+        <v>300</v>
+      </c>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="str">
+      <c r="A7" s="10" t="n">
         <f aca="false">IF(B7="","",ROW()-3)</f>
-        <v/>
-      </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="E7" s="11"/>
       <c r="F7" s="12" t="str">
         <f aca="false">IF(E7="","",IF(E7&lt;10000,"Micro",IF(E7&lt;100000,"Mid","Macro")))</f>
@@ -965,18 +998,26 @@
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
-      <c r="J7" s="13"/>
+      <c r="J7" s="13" t="n">
+        <v>300</v>
+      </c>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="str">
+      <c r="A8" s="10" t="n">
         <f aca="false">IF(B8="","",ROW()-3)</f>
-        <v/>
-      </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="E8" s="11"/>
       <c r="F8" s="12" t="str">
         <f aca="false">IF(E8="","",IF(E8&lt;10000,"Micro",IF(E8&lt;100000,"Mid","Macro")))</f>
@@ -985,18 +1026,26 @@
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
-      <c r="J8" s="13"/>
+      <c r="J8" s="13" t="n">
+        <v>500</v>
+      </c>
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="str">
+      <c r="A9" s="10" t="n">
         <f aca="false">IF(B9="","",ROW()-3)</f>
-        <v/>
-      </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>47</v>
+      </c>
       <c r="E9" s="11"/>
       <c r="F9" s="12" t="str">
         <f aca="false">IF(E9="","",IF(E9&lt;10000,"Micro",IF(E9&lt;100000,"Mid","Macro")))</f>
@@ -1005,18 +1054,26 @@
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
-      <c r="J9" s="13"/>
+      <c r="J9" s="13" t="n">
+        <v>400</v>
+      </c>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="str">
+      <c r="A10" s="10" t="n">
         <f aca="false">IF(B10="","",ROW()-3)</f>
-        <v/>
-      </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
+        <v>7</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>50</v>
+      </c>
       <c r="E10" s="11"/>
       <c r="F10" s="12" t="str">
         <f aca="false">IF(E10="","",IF(E10&lt;10000,"Micro",IF(E10&lt;100000,"Mid","Macro")))</f>
@@ -1025,18 +1082,26 @@
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
-      <c r="J10" s="13"/>
+      <c r="J10" s="13" t="n">
+        <v>200</v>
+      </c>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="str">
+      <c r="A11" s="10" t="n">
         <f aca="false">IF(B11="","",ROW()-3)</f>
-        <v/>
-      </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>53</v>
+      </c>
       <c r="E11" s="11"/>
       <c r="F11" s="12" t="str">
         <f aca="false">IF(E11="","",IF(E11&lt;10000,"Micro",IF(E11&lt;100000,"Mid","Macro")))</f>
@@ -1045,18 +1110,26 @@
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
-      <c r="J11" s="13"/>
+      <c r="J11" s="13" t="n">
+        <v>400</v>
+      </c>
       <c r="K11" s="4"/>
       <c r="L11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="str">
+      <c r="A12" s="10" t="n">
         <f aca="false">IF(B12="","",ROW()-3)</f>
-        <v/>
-      </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>56</v>
+      </c>
       <c r="E12" s="11"/>
       <c r="F12" s="12" t="str">
         <f aca="false">IF(E12="","",IF(E12&lt;10000,"Micro",IF(E12&lt;100000,"Mid","Macro")))</f>
@@ -1065,18 +1138,26 @@
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
-      <c r="J12" s="13"/>
+      <c r="J12" s="13" t="n">
+        <v>400</v>
+      </c>
       <c r="K12" s="4"/>
       <c r="L12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="str">
+      <c r="A13" s="10" t="n">
         <f aca="false">IF(B13="","",ROW()-3)</f>
-        <v/>
-      </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
+        <v>10</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>59</v>
+      </c>
       <c r="E13" s="11"/>
       <c r="F13" s="12" t="str">
         <f aca="false">IF(E13="","",IF(E13&lt;10000,"Micro",IF(E13&lt;100000,"Mid","Macro")))</f>
@@ -1085,18 +1166,26 @@
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="13"/>
+      <c r="J13" s="13" t="n">
+        <v>200</v>
+      </c>
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="str">
+      <c r="A14" s="10" t="n">
         <f aca="false">IF(B14="","",ROW()-3)</f>
-        <v/>
-      </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
+        <v>11</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>62</v>
+      </c>
       <c r="E14" s="11"/>
       <c r="F14" s="12" t="str">
         <f aca="false">IF(E14="","",IF(E14&lt;10000,"Micro",IF(E14&lt;100000,"Mid","Macro")))</f>
@@ -1105,18 +1194,26 @@
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="13"/>
+      <c r="J14" s="13" t="n">
+        <v>700</v>
+      </c>
       <c r="K14" s="4"/>
       <c r="L14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="str">
+      <c r="A15" s="10" t="n">
         <f aca="false">IF(B15="","",ROW()-3)</f>
-        <v/>
-      </c>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
+        <v>12</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="E15" s="11"/>
       <c r="F15" s="12" t="str">
         <f aca="false">IF(E15="","",IF(E15&lt;10000,"Micro",IF(E15&lt;100000,"Mid","Macro")))</f>
@@ -1125,18 +1222,26 @@
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
-      <c r="J15" s="13"/>
+      <c r="J15" s="13" t="n">
+        <v>1000</v>
+      </c>
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="str">
+      <c r="A16" s="10" t="n">
         <f aca="false">IF(B16="","",ROW()-3)</f>
-        <v/>
-      </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
+        <v>13</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>68</v>
+      </c>
       <c r="E16" s="11"/>
       <c r="F16" s="12" t="str">
         <f aca="false">IF(E16="","",IF(E16&lt;10000,"Micro",IF(E16&lt;100000,"Mid","Macro")))</f>
@@ -1145,18 +1250,26 @@
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
-      <c r="J16" s="13"/>
+      <c r="J16" s="13" t="n">
+        <v>200</v>
+      </c>
       <c r="K16" s="4"/>
       <c r="L16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="str">
+      <c r="A17" s="10" t="n">
         <f aca="false">IF(B17="","",ROW()-3)</f>
-        <v/>
-      </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
+        <v>14</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>71</v>
+      </c>
       <c r="E17" s="11"/>
       <c r="F17" s="12" t="str">
         <f aca="false">IF(E17="","",IF(E17&lt;10000,"Micro",IF(E17&lt;100000,"Mid","Macro")))</f>
@@ -1165,7 +1278,9 @@
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
-      <c r="J17" s="13"/>
+      <c r="J17" s="13" t="n">
+        <v>200</v>
+      </c>
       <c r="K17" s="4"/>
       <c r="L17" s="4"/>
     </row>

</xml_diff>

<commit_message>
Add confirmed campaign budget (7k) to Rally x Antseed overview
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P3jSSdGqNpHohJRWxCoL15
</commit_message>
<xml_diff>
--- a/kol-tracker/partners/Rally_x_Antseed_KOL_List.xlsx
+++ b/kol-tracker/partners/Rally_x_Antseed_KOL_List.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
   <si>
     <t xml:space="preserve">Rally x Antseed — KOL Campaign</t>
   </si>
@@ -65,10 +65,13 @@
     <t xml:space="preserve">Combined followers</t>
   </si>
   <si>
-    <t xml:space="preserve">Total budget ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmed budget ($)</t>
+    <t xml:space="preserve">Confirmed campaign budget ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allocated to KOLs ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remaining ($)</t>
   </si>
   <si>
     <t xml:space="preserve">Yellow cells are editable. Followers, region, deliverables and status are pending — fill them in as they get confirmed.</t>
@@ -798,8 +801,7 @@
         <v>14</v>
       </c>
       <c r="C14" s="7" t="n">
-        <f aca="false">SUM('KOL List'!$J$4:$J$200)</f>
-        <v>5400</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -807,13 +809,22 @@
         <v>15</v>
       </c>
       <c r="C15" s="7" t="n">
-        <f aca="false">SUMIF('KOL List'!$K$4:$K$200,"Confirmed",'KOL List'!$J$4:$J$200)</f>
-        <v>0</v>
+        <f aca="false">SUM('KOL List'!$J$4:$J$200)</f>
+        <v>5400</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <f aca="false">C14-C15</f>
+        <v>1600</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -851,45 +862,45 @@
   <sheetData>
     <row r="2" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -898,13 +909,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E4" s="11"/>
       <c r="F4" s="12" t="str">
@@ -926,13 +937,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E5" s="11"/>
       <c r="F5" s="12" t="str">
@@ -954,13 +965,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E6" s="11"/>
       <c r="F6" s="12" t="str">
@@ -982,13 +993,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="12" t="str">
@@ -1010,13 +1021,13 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E8" s="11"/>
       <c r="F8" s="12" t="str">
@@ -1038,13 +1049,13 @@
         <v>6</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E9" s="11"/>
       <c r="F9" s="12" t="str">
@@ -1066,13 +1077,13 @@
         <v>7</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E10" s="11"/>
       <c r="F10" s="12" t="str">
@@ -1094,13 +1105,13 @@
         <v>8</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E11" s="11"/>
       <c r="F11" s="12" t="str">
@@ -1122,13 +1133,13 @@
         <v>9</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E12" s="11"/>
       <c r="F12" s="12" t="str">
@@ -1150,13 +1161,13 @@
         <v>10</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E13" s="11"/>
       <c r="F13" s="12" t="str">
@@ -1178,13 +1189,13 @@
         <v>11</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E14" s="11"/>
       <c r="F14" s="12" t="str">
@@ -1206,13 +1217,13 @@
         <v>12</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E15" s="11"/>
       <c r="F15" s="12" t="str">
@@ -1234,13 +1245,13 @@
         <v>13</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E16" s="11"/>
       <c r="F16" s="12" t="str">
@@ -1262,13 +1273,13 @@
         <v>14</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E17" s="11"/>
       <c r="F17" s="12" t="str">

</xml_diff>